<commit_message>
ci(dev): publish dev build from 1347e2174cc189bad009ff3cebb5ad9b96bb2154 1347e2174cc189bad009ff3cebb5ad9b96bb2154
</commit_message>
<xml_diff>
--- a/dev/StructureDefinition-ph-core-encounter.xlsx
+++ b/dev/StructureDefinition-ph-core-encounter.xlsx
@@ -9,11 +9,14 @@
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AN$78</definedName>
+  </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2676" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2820" uniqueCount="486">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-23T13:24:52+00:00</t>
+    <t>2026-03-25T02:48:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -748,7 +751,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-patient)
+    <t xml:space="preserve">Reference(http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-patient|Group)
 </t>
   </si>
   <si>
@@ -887,7 +890,7 @@
     <t>Encounter.participant.individual</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-practitioner|PractitionerRole|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-relatedperson)
+    <t xml:space="preserve">Reference(http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-practitioner|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-relatedperson|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-practitionerrole)
 </t>
   </si>
   <si>
@@ -952,6 +955,75 @@
     <t>PV1-44, PV1-45</t>
   </si>
   <si>
+    <t>Encounter.period.id</t>
+  </si>
+  <si>
+    <t>Encounter.period.extension</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value:url}
+</t>
+  </si>
+  <si>
+    <t>Extensions are always sliced by (at least) url</t>
+  </si>
+  <si>
+    <t>open</t>
+  </si>
+  <si>
+    <t>Encounter.period.start</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dateTime
+</t>
+  </si>
+  <si>
+    <t>Starting time with inclusive boundary</t>
+  </si>
+  <si>
+    <t>The start of the period. The boundary is inclusive.</t>
+  </si>
+  <si>
+    <t>If the low element is missing, the meaning is that the low boundary is not known.</t>
+  </si>
+  <si>
+    <t>Period.start</t>
+  </si>
+  <si>
+    <t xml:space="preserve">per-1
+</t>
+  </si>
+  <si>
+    <t>./low</t>
+  </si>
+  <si>
+    <t>DR.1</t>
+  </si>
+  <si>
+    <t>Encounter.period.end</t>
+  </si>
+  <si>
+    <t>End time with inclusive boundary, if not ongoing</t>
+  </si>
+  <si>
+    <t>The end of the period. If the end of the period is missing, it means no end was known or planned at the time the instance was created. The start may be in the past, and the end date in the future, which means that period is expected/planned to end at that time.</t>
+  </si>
+  <si>
+    <t>The high value includes any matching date/time. i.e. 2012-02-03T10:00:00 is in a period that has an end value of 2012-02-03.</t>
+  </si>
+  <si>
+    <t>If the end of the period is missing, it means that the period is ongoing</t>
+  </si>
+  <si>
+    <t>Period.end</t>
+  </si>
+  <si>
+    <t>./high</t>
+  </si>
+  <si>
+    <t>DR.2</t>
+  </si>
+  <si>
     <t>Encounter.length</t>
   </si>
   <si>
@@ -1011,7 +1083,7 @@
     <t>Encounter.reasonReference</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Condition|4.0.1|Procedure|4.0.1|Observation|4.0.1|ImmunizationRecommendation|4.0.1)
+    <t xml:space="preserve">Reference(Condition|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-observation|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-procedure|ImmunizationRecommendation)
 </t>
   </si>
   <si>
@@ -1046,7 +1118,7 @@
 discharge diagnosisindication</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Condition|4.0.1|Procedure|4.0.1)
+    <t xml:space="preserve">Reference(Condition|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-procedure)
 </t>
   </si>
   <si>
@@ -1156,130 +1228,134 @@
     <t>Encounter.hospitalization.origin</t>
   </si>
   <si>
+    <t xml:space="preserve">Reference(http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-location|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-organization)
+</t>
+  </si>
+  <si>
+    <t>The location/organization from which the patient came before admission</t>
+  </si>
+  <si>
+    <t>The location/organization from which the patient came before admission.</t>
+  </si>
+  <si>
+    <t>.participation[typeCode=ORG].role</t>
+  </si>
+  <si>
+    <t>Encounter.hospitalization.admitSource</t>
+  </si>
+  <si>
+    <t>From where patient was admitted (physician referral, transfer)</t>
+  </si>
+  <si>
+    <t>From where patient was admitted (physician referral, transfer).</t>
+  </si>
+  <si>
+    <t>From where the patient was admitted.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/encounter-admit-source|4.0.1</t>
+  </si>
+  <si>
+    <t>.admissionReferralSourceCode</t>
+  </si>
+  <si>
+    <t>PV1-14</t>
+  </si>
+  <si>
+    <t>Encounter.hospitalization.reAdmission</t>
+  </si>
+  <si>
+    <t>The type of hospital re-admission that has occurred (if any). If the value is absent, then this is not identified as a readmission</t>
+  </si>
+  <si>
+    <t>Whether this hospitalization is a readmission and why if known.</t>
+  </si>
+  <si>
+    <t>The reason for re-admission of this hospitalization encounter.</t>
+  </si>
+  <si>
+    <t>http://terminology.hl7.org/ValueSet/v2-0092</t>
+  </si>
+  <si>
+    <t>PV1-13</t>
+  </si>
+  <si>
+    <t>Encounter.hospitalization.dietPreference</t>
+  </si>
+  <si>
+    <t>Diet preferences reported by the patient</t>
+  </si>
+  <si>
+    <t>Diet preferences reported by the patient.</t>
+  </si>
+  <si>
+    <t>For example, a patient may request both a dairy-free and nut-free diet preference (not mutually exclusive).</t>
+  </si>
+  <si>
+    <t>Used to track patient's diet restrictions and/or preference. For a complete description of the nutrition needs of a patient during their stay, one should use the nutritionOrder resource which links to Encounter.</t>
+  </si>
+  <si>
+    <t>Medical, cultural or ethical food preferences to help with catering requirements.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/encounter-diet|4.0.1</t>
+  </si>
+  <si>
+    <t>.outboundRelationship[typeCode=COMP].target[classCode=SBADM, moodCode=EVN, code="diet"]</t>
+  </si>
+  <si>
+    <t>PV1-38</t>
+  </si>
+  <si>
+    <t>Encounter.hospitalization.specialCourtesy</t>
+  </si>
+  <si>
+    <t>Special courtesies (VIP, board member)</t>
+  </si>
+  <si>
+    <t>Special courtesies (VIP, board member).</t>
+  </si>
+  <si>
+    <t>Special courtesies.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/encounter-special-courtesy|4.0.1</t>
+  </si>
+  <si>
+    <t>.specialCourtesiesCode</t>
+  </si>
+  <si>
+    <t>PV1-16</t>
+  </si>
+  <si>
+    <t>Encounter.hospitalization.specialArrangement</t>
+  </si>
+  <si>
+    <t>Wheelchair, translator, stretcher, etc.</t>
+  </si>
+  <si>
+    <t>Any special requests that have been made for this hospitalization encounter, such as the provision of specific equipment or other things.</t>
+  </si>
+  <si>
+    <t>Special arrangements.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/encounter-special-arrangements|4.0.1</t>
+  </si>
+  <si>
+    <t>.specialArrangementCode</t>
+  </si>
+  <si>
+    <t>PV1-15 / OBR-30 / OBR-43</t>
+  </si>
+  <si>
+    <t>Encounter.hospitalization.destination</t>
+  </si>
+  <si>
     <t xml:space="preserve">Reference(Location|4.0.1|Organization|4.0.1)
 </t>
   </si>
   <si>
-    <t>The location/organization from which the patient came before admission</t>
-  </si>
-  <si>
-    <t>The location/organization from which the patient came before admission.</t>
-  </si>
-  <si>
-    <t>.participation[typeCode=ORG].role</t>
-  </si>
-  <si>
-    <t>Encounter.hospitalization.admitSource</t>
-  </si>
-  <si>
-    <t>From where patient was admitted (physician referral, transfer)</t>
-  </si>
-  <si>
-    <t>From where patient was admitted (physician referral, transfer).</t>
-  </si>
-  <si>
-    <t>From where the patient was admitted.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/encounter-admit-source|4.0.1</t>
-  </si>
-  <si>
-    <t>.admissionReferralSourceCode</t>
-  </si>
-  <si>
-    <t>PV1-14</t>
-  </si>
-  <si>
-    <t>Encounter.hospitalization.reAdmission</t>
-  </si>
-  <si>
-    <t>The type of hospital re-admission that has occurred (if any). If the value is absent, then this is not identified as a readmission</t>
-  </si>
-  <si>
-    <t>Whether this hospitalization is a readmission and why if known.</t>
-  </si>
-  <si>
-    <t>The reason for re-admission of this hospitalization encounter.</t>
-  </si>
-  <si>
-    <t>http://terminology.hl7.org/ValueSet/v2-0092</t>
-  </si>
-  <si>
-    <t>PV1-13</t>
-  </si>
-  <si>
-    <t>Encounter.hospitalization.dietPreference</t>
-  </si>
-  <si>
-    <t>Diet preferences reported by the patient</t>
-  </si>
-  <si>
-    <t>Diet preferences reported by the patient.</t>
-  </si>
-  <si>
-    <t>For example, a patient may request both a dairy-free and nut-free diet preference (not mutually exclusive).</t>
-  </si>
-  <si>
-    <t>Used to track patient's diet restrictions and/or preference. For a complete description of the nutrition needs of a patient during their stay, one should use the nutritionOrder resource which links to Encounter.</t>
-  </si>
-  <si>
-    <t>Medical, cultural or ethical food preferences to help with catering requirements.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/encounter-diet|4.0.1</t>
-  </si>
-  <si>
-    <t>.outboundRelationship[typeCode=COMP].target[classCode=SBADM, moodCode=EVN, code="diet"]</t>
-  </si>
-  <si>
-    <t>PV1-38</t>
-  </si>
-  <si>
-    <t>Encounter.hospitalization.specialCourtesy</t>
-  </si>
-  <si>
-    <t>Special courtesies (VIP, board member)</t>
-  </si>
-  <si>
-    <t>Special courtesies (VIP, board member).</t>
-  </si>
-  <si>
-    <t>Special courtesies.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/encounter-special-courtesy|4.0.1</t>
-  </si>
-  <si>
-    <t>.specialCourtesiesCode</t>
-  </si>
-  <si>
-    <t>PV1-16</t>
-  </si>
-  <si>
-    <t>Encounter.hospitalization.specialArrangement</t>
-  </si>
-  <si>
-    <t>Wheelchair, translator, stretcher, etc.</t>
-  </si>
-  <si>
-    <t>Any special requests that have been made for this hospitalization encounter, such as the provision of specific equipment or other things.</t>
-  </si>
-  <si>
-    <t>Special arrangements.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/encounter-special-arrangements|4.0.1</t>
-  </si>
-  <si>
-    <t>.specialArrangementCode</t>
-  </si>
-  <si>
-    <t>PV1-15 / OBR-30 / OBR-43</t>
-  </si>
-  <si>
-    <t>Encounter.hospitalization.destination</t>
-  </si>
-  <si>
     <t>Location/organization to which the patient is discharged</t>
   </si>
   <si>
@@ -1340,7 +1416,7 @@
     <t>Encounter.location.location</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Location|4.0.1)
+    <t xml:space="preserve">Reference(http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-location)
 </t>
   </si>
   <si>
@@ -1411,7 +1487,7 @@
     <t>Encounter.serviceProvider</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Organization|4.0.1)
+    <t xml:space="preserve">Reference(http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-organization)
 </t>
   </si>
   <si>
@@ -1577,6 +1653,21 @@
       <alignment vertical="top" wrapText="true"/>
     </xf>
   </cellXfs>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor indexed="22"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color indexed="22"/>
+        <i val="true"/>
+      </font>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
@@ -1750,7 +1841,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AN74"/>
+  <dimension ref="A1:AN78"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="39.16015625" customWidth="true" bestFit="true"/>
@@ -1763,7 +1854,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="135.7421875" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="181.2734375" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -1781,7 +1872,7 @@
     <col min="26" max="26" width="52.75390625" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="32" max="32" width="39.16015625" customWidth="true" bestFit="true" hidden="true"/>
@@ -1916,7 +2007,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" hidden="true">
       <c r="A2" t="s" s="2">
         <v>30</v>
       </c>
@@ -2028,7 +2119,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" hidden="true">
       <c r="A3" t="s" s="2">
         <v>87</v>
       </c>
@@ -2142,7 +2233,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" hidden="true">
       <c r="A4" t="s" s="2">
         <v>95</v>
       </c>
@@ -2254,7 +2345,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" hidden="true">
       <c r="A5" t="s" s="2">
         <v>101</v>
       </c>
@@ -2368,7 +2459,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" hidden="true">
       <c r="A6" t="s" s="2">
         <v>107</v>
       </c>
@@ -2482,7 +2573,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" hidden="true">
       <c r="A7" t="s" s="2">
         <v>116</v>
       </c>
@@ -2596,7 +2687,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" hidden="true">
       <c r="A8" t="s" s="2">
         <v>124</v>
       </c>
@@ -2710,7 +2801,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" hidden="true">
       <c r="A9" t="s" s="2">
         <v>132</v>
       </c>
@@ -2824,7 +2915,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" hidden="true">
       <c r="A10" t="s" s="2">
         <v>140</v>
       </c>
@@ -2959,7 +3050,7 @@
         <v>79</v>
       </c>
       <c r="H11" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I11" t="s" s="2">
         <v>80</v>
@@ -3071,7 +3162,7 @@
         <v>88</v>
       </c>
       <c r="H12" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I12" t="s" s="2">
         <v>89</v>
@@ -3166,7 +3257,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" hidden="true">
       <c r="A13" t="s" s="2">
         <v>164</v>
       </c>
@@ -3280,7 +3371,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
         <v>170</v>
       </c>
@@ -3392,7 +3483,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
         <v>175</v>
       </c>
@@ -3506,7 +3597,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
         <v>178</v>
       </c>
@@ -3622,7 +3713,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
         <v>183</v>
       </c>
@@ -3734,7 +3825,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
         <v>184</v>
       </c>
@@ -3865,7 +3956,7 @@
         <v>88</v>
       </c>
       <c r="H19" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I19" t="s" s="2">
         <v>80</v>
@@ -3958,7 +4049,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
         <v>198</v>
       </c>
@@ -4070,7 +4161,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
         <v>201</v>
       </c>
@@ -4182,7 +4273,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
         <v>202</v>
       </c>
@@ -4296,7 +4387,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
         <v>203</v>
       </c>
@@ -4412,7 +4503,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
         <v>204</v>
       </c>
@@ -4524,7 +4615,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
         <v>207</v>
       </c>
@@ -4655,7 +4746,7 @@
         <v>79</v>
       </c>
       <c r="H26" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I26" t="s" s="2">
         <v>80</v>
@@ -4750,7 +4841,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
         <v>221</v>
       </c>
@@ -4862,7 +4953,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
         <v>227</v>
       </c>
@@ -4987,13 +5078,13 @@
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G29" t="s" s="2">
         <v>88</v>
       </c>
       <c r="H29" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I29" t="s" s="2">
         <v>80</v>
@@ -5088,7 +5179,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
         <v>244</v>
       </c>
@@ -5200,7 +5291,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
         <v>251</v>
       </c>
@@ -5331,7 +5422,7 @@
         <v>79</v>
       </c>
       <c r="H32" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I32" t="s" s="2">
         <v>80</v>
@@ -5424,7 +5515,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
         <v>264</v>
       </c>
@@ -5536,7 +5627,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
         <v>265</v>
       </c>
@@ -5650,7 +5741,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
         <v>266</v>
       </c>
@@ -5785,7 +5876,7 @@
         <v>79</v>
       </c>
       <c r="H36" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I36" t="s" s="2">
         <v>80</v>
@@ -5880,7 +5971,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
         <v>275</v>
       </c>
@@ -5992,7 +6083,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
         <v>280</v>
       </c>
@@ -6104,7 +6195,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
         <v>288</v>
       </c>
@@ -6235,7 +6326,7 @@
         <v>88</v>
       </c>
       <c r="H40" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I40" t="s" s="2">
         <v>80</v>
@@ -6330,7 +6421,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
         <v>302</v>
       </c>
@@ -6358,17 +6449,15 @@
         <v>80</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>303</v>
+        <v>171</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>304</v>
+        <v>172</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>305</v>
-      </c>
-      <c r="N41" t="s" s="2">
-        <v>306</v>
-      </c>
+        <v>173</v>
+      </c>
+      <c r="N41" s="2"/>
       <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
         <v>80</v>
@@ -6417,7 +6506,7 @@
         <v>80</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>302</v>
+        <v>174</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>78</v>
@@ -6429,31 +6518,31 @@
         <v>80</v>
       </c>
       <c r="AJ41" t="s" s="2">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>298</v>
+        <v>80</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>307</v>
+        <v>169</v>
       </c>
       <c r="AM41" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN41" t="s" s="2">
-        <v>308</v>
+        <v>80</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
-        <v>310</v>
+        <v>133</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
@@ -6469,19 +6558,19 @@
         <v>80</v>
       </c>
       <c r="J42" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>211</v>
+        <v>134</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>311</v>
+        <v>135</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>312</v>
+        <v>176</v>
       </c>
       <c r="N42" t="s" s="2">
-        <v>313</v>
+        <v>137</v>
       </c>
       <c r="O42" s="2"/>
       <c r="P42" t="s" s="2">
@@ -6507,31 +6596,31 @@
         <v>80</v>
       </c>
       <c r="X42" t="s" s="2">
-        <v>112</v>
+        <v>80</v>
       </c>
       <c r="Y42" t="s" s="2">
-        <v>314</v>
+        <v>80</v>
       </c>
       <c r="Z42" t="s" s="2">
-        <v>315</v>
+        <v>80</v>
       </c>
       <c r="AA42" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AB42" t="s" s="2">
-        <v>80</v>
+        <v>304</v>
       </c>
       <c r="AC42" t="s" s="2">
-        <v>80</v>
+        <v>305</v>
       </c>
       <c r="AD42" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE42" t="s" s="2">
-        <v>80</v>
+        <v>306</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>309</v>
+        <v>177</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>78</v>
@@ -6543,41 +6632,41 @@
         <v>80</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>316</v>
+        <v>80</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>317</v>
+        <v>169</v>
       </c>
       <c r="AM42" t="s" s="2">
-        <v>318</v>
+        <v>80</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>319</v>
+        <v>80</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>320</v>
+        <v>307</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>320</v>
+        <v>307</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>310</v>
+        <v>80</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G43" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H43" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I43" t="s" s="2">
         <v>80</v>
@@ -6586,16 +6675,16 @@
         <v>89</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>321</v>
+        <v>308</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>322</v>
+        <v>309</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="N43" t="s" s="2">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
@@ -6645,39 +6734,39 @@
         <v>80</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH43" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI43" t="s" s="2">
-        <v>80</v>
+        <v>313</v>
       </c>
       <c r="AJ43" t="s" s="2">
         <v>100</v>
       </c>
       <c r="AK43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL43" t="s" s="2">
+        <v>314</v>
+      </c>
+      <c r="AM43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN43" t="s" s="2">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="44" hidden="true">
+      <c r="A44" t="s" s="2">
         <v>316</v>
       </c>
-      <c r="AL43" t="s" s="2">
-        <v>317</v>
-      </c>
-      <c r="AM43" t="s" s="2">
-        <v>318</v>
-      </c>
-      <c r="AN43" t="s" s="2">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="s" s="2">
-        <v>323</v>
-      </c>
       <c r="B44" t="s" s="2">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6688,7 +6777,7 @@
         <v>78</v>
       </c>
       <c r="G44" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H44" t="s" s="2">
         <v>80</v>
@@ -6700,20 +6789,24 @@
         <v>89</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>165</v>
+        <v>308</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>325</v>
-      </c>
-      <c r="N44" s="2"/>
+        <v>318</v>
+      </c>
+      <c r="N44" t="s" s="2">
+        <v>319</v>
+      </c>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="Q44" s="2"/>
+      <c r="Q44" t="s" s="2">
+        <v>320</v>
+      </c>
       <c r="R44" t="s" s="2">
         <v>80</v>
       </c>
@@ -6757,16 +6850,16 @@
         <v>80</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH44" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI44" t="s" s="2">
-        <v>80</v>
+        <v>313</v>
       </c>
       <c r="AJ44" t="s" s="2">
         <v>100</v>
@@ -6775,21 +6868,21 @@
         <v>80</v>
       </c>
       <c r="AL44" t="s" s="2">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="AM44" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN44" t="s" s="2">
-        <v>80</v>
+        <v>323</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6812,15 +6905,17 @@
         <v>80</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>171</v>
+        <v>325</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>172</v>
+        <v>326</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>173</v>
-      </c>
-      <c r="N45" s="2"/>
+        <v>327</v>
+      </c>
+      <c r="N45" t="s" s="2">
+        <v>328</v>
+      </c>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
         <v>80</v>
@@ -6869,7 +6964,7 @@
         <v>80</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>174</v>
+        <v>324</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>78</v>
@@ -6881,31 +6976,31 @@
         <v>80</v>
       </c>
       <c r="AJ45" t="s" s="2">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="AK45" t="s" s="2">
-        <v>80</v>
+        <v>298</v>
       </c>
       <c r="AL45" t="s" s="2">
-        <v>169</v>
+        <v>329</v>
       </c>
       <c r="AM45" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN45" t="s" s="2">
-        <v>80</v>
+        <v>330</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
-        <v>133</v>
+        <v>332</v>
       </c>
       <c r="E46" s="2"/>
       <c r="F46" t="s" s="2">
@@ -6915,25 +7010,25 @@
         <v>79</v>
       </c>
       <c r="H46" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I46" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J46" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>134</v>
+        <v>211</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>135</v>
+        <v>333</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>176</v>
+        <v>334</v>
       </c>
       <c r="N46" t="s" s="2">
-        <v>137</v>
+        <v>335</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
@@ -6959,13 +7054,13 @@
         <v>80</v>
       </c>
       <c r="X46" t="s" s="2">
-        <v>80</v>
+        <v>112</v>
       </c>
       <c r="Y46" t="s" s="2">
-        <v>80</v>
+        <v>336</v>
       </c>
       <c r="Z46" t="s" s="2">
-        <v>80</v>
+        <v>337</v>
       </c>
       <c r="AA46" t="s" s="2">
         <v>80</v>
@@ -6983,7 +7078,7 @@
         <v>80</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>177</v>
+        <v>331</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>78</v>
@@ -6995,31 +7090,31 @@
         <v>80</v>
       </c>
       <c r="AJ46" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK46" t="s" s="2">
-        <v>80</v>
+        <v>338</v>
       </c>
       <c r="AL46" t="s" s="2">
-        <v>169</v>
+        <v>339</v>
       </c>
       <c r="AM46" t="s" s="2">
-        <v>80</v>
+        <v>340</v>
       </c>
       <c r="AN46" t="s" s="2">
-        <v>80</v>
+        <v>341</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>329</v>
+        <v>342</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>329</v>
+        <v>342</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
-        <v>179</v>
+        <v>332</v>
       </c>
       <c r="E47" s="2"/>
       <c r="F47" t="s" s="2">
@@ -7029,29 +7124,27 @@
         <v>79</v>
       </c>
       <c r="H47" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I47" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="J47" t="s" s="2">
         <v>89</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>134</v>
+        <v>343</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>180</v>
+        <v>344</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>181</v>
+        <v>334</v>
       </c>
       <c r="N47" t="s" s="2">
-        <v>137</v>
-      </c>
-      <c r="O47" t="s" s="2">
-        <v>143</v>
-      </c>
+        <v>335</v>
+      </c>
+      <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
         <v>80</v>
       </c>
@@ -7099,7 +7192,7 @@
         <v>80</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>182</v>
+        <v>342</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>78</v>
@@ -7111,38 +7204,38 @@
         <v>80</v>
       </c>
       <c r="AJ47" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK47" t="s" s="2">
-        <v>80</v>
+        <v>338</v>
       </c>
       <c r="AL47" t="s" s="2">
-        <v>131</v>
+        <v>339</v>
       </c>
       <c r="AM47" t="s" s="2">
-        <v>80</v>
+        <v>340</v>
       </c>
       <c r="AN47" t="s" s="2">
-        <v>80</v>
+        <v>341</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>330</v>
+        <v>345</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>330</v>
+        <v>345</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
-        <v>331</v>
+        <v>80</v>
       </c>
       <c r="E48" s="2"/>
       <c r="F48" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G48" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H48" t="s" s="2">
         <v>80</v>
@@ -7154,17 +7247,15 @@
         <v>89</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>332</v>
+        <v>165</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>333</v>
+        <v>346</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>334</v>
-      </c>
-      <c r="N48" t="s" s="2">
-        <v>313</v>
-      </c>
+        <v>347</v>
+      </c>
+      <c r="N48" s="2"/>
       <c r="O48" s="2"/>
       <c r="P48" t="s" s="2">
         <v>80</v>
@@ -7213,13 +7304,13 @@
         <v>80</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>330</v>
+        <v>345</v>
       </c>
       <c r="AG48" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="AH48" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI48" t="s" s="2">
         <v>80</v>
@@ -7228,24 +7319,24 @@
         <v>100</v>
       </c>
       <c r="AK48" t="s" s="2">
-        <v>335</v>
+        <v>80</v>
       </c>
       <c r="AL48" t="s" s="2">
-        <v>336</v>
+        <v>348</v>
       </c>
       <c r="AM48" t="s" s="2">
-        <v>318</v>
+        <v>80</v>
       </c>
       <c r="AN48" t="s" s="2">
-        <v>337</v>
+        <v>80</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>338</v>
+        <v>349</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>338</v>
+        <v>349</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7268,13 +7359,13 @@
         <v>80</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>211</v>
+        <v>171</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>339</v>
+        <v>172</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>340</v>
+        <v>173</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
@@ -7301,13 +7392,13 @@
         <v>80</v>
       </c>
       <c r="X49" t="s" s="2">
-        <v>112</v>
+        <v>80</v>
       </c>
       <c r="Y49" t="s" s="2">
-        <v>341</v>
+        <v>80</v>
       </c>
       <c r="Z49" t="s" s="2">
-        <v>342</v>
+        <v>80</v>
       </c>
       <c r="AA49" t="s" s="2">
         <v>80</v>
@@ -7325,7 +7416,7 @@
         <v>80</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>338</v>
+        <v>174</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>78</v>
@@ -7337,7 +7428,7 @@
         <v>80</v>
       </c>
       <c r="AJ49" t="s" s="2">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AK49" t="s" s="2">
         <v>80</v>
@@ -7352,23 +7443,23 @@
         <v>80</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
-        <v>80</v>
+        <v>133</v>
       </c>
       <c r="E50" s="2"/>
       <c r="F50" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G50" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H50" t="s" s="2">
         <v>80</v>
@@ -7380,15 +7471,17 @@
         <v>80</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>344</v>
+        <v>134</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>345</v>
+        <v>135</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>346</v>
-      </c>
-      <c r="N50" s="2"/>
+        <v>176</v>
+      </c>
+      <c r="N50" t="s" s="2">
+        <v>137</v>
+      </c>
       <c r="O50" s="2"/>
       <c r="P50" t="s" s="2">
         <v>80</v>
@@ -7437,25 +7530,25 @@
         <v>80</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>343</v>
+        <v>177</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH50" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI50" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ50" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK50" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL50" t="s" s="2">
-        <v>347</v>
+        <v>169</v>
       </c>
       <c r="AM50" t="s" s="2">
         <v>80</v>
@@ -7464,16 +7557,16 @@
         <v>80</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
-        <v>80</v>
+        <v>179</v>
       </c>
       <c r="E51" s="2"/>
       <c r="F51" t="s" s="2">
@@ -7486,24 +7579,26 @@
         <v>80</v>
       </c>
       <c r="I51" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="J51" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>349</v>
+        <v>134</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>350</v>
+        <v>180</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>351</v>
+        <v>181</v>
       </c>
       <c r="N51" t="s" s="2">
-        <v>352</v>
-      </c>
-      <c r="O51" s="2"/>
+        <v>137</v>
+      </c>
+      <c r="O51" t="s" s="2">
+        <v>143</v>
+      </c>
       <c r="P51" t="s" s="2">
         <v>80</v>
       </c>
@@ -7551,7 +7646,7 @@
         <v>80</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>348</v>
+        <v>182</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>78</v>
@@ -7563,13 +7658,13 @@
         <v>80</v>
       </c>
       <c r="AJ51" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK51" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL51" t="s" s="2">
-        <v>353</v>
+        <v>131</v>
       </c>
       <c r="AM51" t="s" s="2">
         <v>80</v>
@@ -7578,20 +7673,20 @@
         <v>80</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
-        <v>80</v>
+        <v>353</v>
       </c>
       <c r="E52" s="2"/>
       <c r="F52" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G52" t="s" s="2">
         <v>88</v>
@@ -7603,10 +7698,10 @@
         <v>80</v>
       </c>
       <c r="J52" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>165</v>
+        <v>354</v>
       </c>
       <c r="L52" t="s" s="2">
         <v>355</v>
@@ -7615,7 +7710,7 @@
         <v>356</v>
       </c>
       <c r="N52" t="s" s="2">
-        <v>357</v>
+        <v>335</v>
       </c>
       <c r="O52" s="2"/>
       <c r="P52" t="s" s="2">
@@ -7665,10 +7760,10 @@
         <v>80</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="AG52" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="AH52" t="s" s="2">
         <v>88</v>
@@ -7680,24 +7775,24 @@
         <v>100</v>
       </c>
       <c r="AK52" t="s" s="2">
-        <v>80</v>
+        <v>357</v>
       </c>
       <c r="AL52" t="s" s="2">
         <v>358</v>
       </c>
       <c r="AM52" t="s" s="2">
-        <v>80</v>
+        <v>340</v>
       </c>
       <c r="AN52" t="s" s="2">
-        <v>80</v>
+        <v>359</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -7720,13 +7815,13 @@
         <v>80</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>171</v>
+        <v>211</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>172</v>
+        <v>361</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>173</v>
+        <v>362</v>
       </c>
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
@@ -7753,13 +7848,13 @@
         <v>80</v>
       </c>
       <c r="X53" t="s" s="2">
-        <v>80</v>
+        <v>112</v>
       </c>
       <c r="Y53" t="s" s="2">
-        <v>80</v>
+        <v>363</v>
       </c>
       <c r="Z53" t="s" s="2">
-        <v>80</v>
+        <v>364</v>
       </c>
       <c r="AA53" t="s" s="2">
         <v>80</v>
@@ -7777,7 +7872,7 @@
         <v>80</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>174</v>
+        <v>360</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>78</v>
@@ -7789,7 +7884,7 @@
         <v>80</v>
       </c>
       <c r="AJ53" t="s" s="2">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="AK53" t="s" s="2">
         <v>80</v>
@@ -7804,23 +7899,23 @@
         <v>80</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
-        <v>133</v>
+        <v>80</v>
       </c>
       <c r="E54" s="2"/>
       <c r="F54" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G54" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H54" t="s" s="2">
         <v>80</v>
@@ -7832,17 +7927,15 @@
         <v>80</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>134</v>
+        <v>366</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>135</v>
+        <v>367</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>176</v>
-      </c>
-      <c r="N54" t="s" s="2">
-        <v>137</v>
-      </c>
+        <v>368</v>
+      </c>
+      <c r="N54" s="2"/>
       <c r="O54" s="2"/>
       <c r="P54" t="s" s="2">
         <v>80</v>
@@ -7891,25 +7984,25 @@
         <v>80</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>177</v>
+        <v>365</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH54" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI54" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ54" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK54" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL54" t="s" s="2">
-        <v>169</v>
+        <v>369</v>
       </c>
       <c r="AM54" t="s" s="2">
         <v>80</v>
@@ -7918,16 +8011,16 @@
         <v>80</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>361</v>
+        <v>370</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>361</v>
+        <v>370</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
-        <v>179</v>
+        <v>80</v>
       </c>
       <c r="E55" s="2"/>
       <c r="F55" t="s" s="2">
@@ -7940,26 +8033,24 @@
         <v>80</v>
       </c>
       <c r="I55" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="J55" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>134</v>
+        <v>371</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>180</v>
+        <v>372</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>181</v>
+        <v>373</v>
       </c>
       <c r="N55" t="s" s="2">
-        <v>137</v>
-      </c>
-      <c r="O55" t="s" s="2">
-        <v>143</v>
-      </c>
+        <v>374</v>
+      </c>
+      <c r="O55" s="2"/>
       <c r="P55" t="s" s="2">
         <v>80</v>
       </c>
@@ -8007,7 +8098,7 @@
         <v>80</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>182</v>
+        <v>370</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>78</v>
@@ -8019,13 +8110,13 @@
         <v>80</v>
       </c>
       <c r="AJ55" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK55" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL55" t="s" s="2">
-        <v>131</v>
+        <v>375</v>
       </c>
       <c r="AM55" t="s" s="2">
         <v>80</v>
@@ -8036,10 +8127,10 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>362</v>
+        <v>376</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>362</v>
+        <v>376</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -8053,7 +8144,7 @@
         <v>88</v>
       </c>
       <c r="H56" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I56" t="s" s="2">
         <v>80</v>
@@ -8062,15 +8153,17 @@
         <v>80</v>
       </c>
       <c r="K56" t="s" s="2">
-        <v>146</v>
+        <v>165</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>363</v>
+        <v>377</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>364</v>
-      </c>
-      <c r="N56" s="2"/>
+        <v>378</v>
+      </c>
+      <c r="N56" t="s" s="2">
+        <v>379</v>
+      </c>
       <c r="O56" s="2"/>
       <c r="P56" t="s" s="2">
         <v>80</v>
@@ -8119,7 +8212,7 @@
         <v>80</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>362</v>
+        <v>376</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>78</v>
@@ -8137,21 +8230,21 @@
         <v>80</v>
       </c>
       <c r="AL56" t="s" s="2">
-        <v>150</v>
+        <v>380</v>
       </c>
       <c r="AM56" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN56" t="s" s="2">
-        <v>365</v>
+        <v>80</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>366</v>
+        <v>381</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>366</v>
+        <v>381</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -8174,13 +8267,13 @@
         <v>80</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>367</v>
+        <v>171</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>368</v>
+        <v>172</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>369</v>
+        <v>173</v>
       </c>
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
@@ -8231,7 +8324,7 @@
         <v>80</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>366</v>
+        <v>174</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>78</v>
@@ -8243,13 +8336,13 @@
         <v>80</v>
       </c>
       <c r="AJ57" t="s" s="2">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AK57" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL57" t="s" s="2">
-        <v>370</v>
+        <v>169</v>
       </c>
       <c r="AM57" t="s" s="2">
         <v>80</v>
@@ -8258,23 +8351,23 @@
         <v>80</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
-        <v>80</v>
+        <v>133</v>
       </c>
       <c r="E58" s="2"/>
       <c r="F58" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G58" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H58" t="s" s="2">
         <v>80</v>
@@ -8286,15 +8379,17 @@
         <v>80</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>211</v>
+        <v>134</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>372</v>
+        <v>135</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>373</v>
-      </c>
-      <c r="N58" s="2"/>
+        <v>176</v>
+      </c>
+      <c r="N58" t="s" s="2">
+        <v>137</v>
+      </c>
       <c r="O58" s="2"/>
       <c r="P58" t="s" s="2">
         <v>80</v>
@@ -8319,13 +8414,13 @@
         <v>80</v>
       </c>
       <c r="X58" t="s" s="2">
-        <v>112</v>
+        <v>80</v>
       </c>
       <c r="Y58" t="s" s="2">
-        <v>374</v>
+        <v>80</v>
       </c>
       <c r="Z58" t="s" s="2">
-        <v>375</v>
+        <v>80</v>
       </c>
       <c r="AA58" t="s" s="2">
         <v>80</v>
@@ -8343,71 +8438,75 @@
         <v>80</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>371</v>
+        <v>177</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH58" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI58" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ58" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK58" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL58" t="s" s="2">
-        <v>376</v>
+        <v>169</v>
       </c>
       <c r="AM58" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN58" t="s" s="2">
-        <v>377</v>
+        <v>80</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
-        <v>80</v>
+        <v>179</v>
       </c>
       <c r="E59" s="2"/>
       <c r="F59" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G59" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H59" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I59" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="J59" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>211</v>
+        <v>134</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>379</v>
+        <v>180</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>380</v>
-      </c>
-      <c r="N59" s="2"/>
-      <c r="O59" s="2"/>
+        <v>181</v>
+      </c>
+      <c r="N59" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="O59" t="s" s="2">
+        <v>143</v>
+      </c>
       <c r="P59" t="s" s="2">
         <v>80</v>
       </c>
@@ -8431,13 +8530,13 @@
         <v>80</v>
       </c>
       <c r="X59" t="s" s="2">
-        <v>215</v>
+        <v>80</v>
       </c>
       <c r="Y59" t="s" s="2">
-        <v>381</v>
+        <v>80</v>
       </c>
       <c r="Z59" t="s" s="2">
-        <v>382</v>
+        <v>80</v>
       </c>
       <c r="AA59" t="s" s="2">
         <v>80</v>
@@ -8455,34 +8554,34 @@
         <v>80</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>378</v>
+        <v>182</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH59" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI59" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ59" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK59" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL59" t="s" s="2">
-        <v>169</v>
+        <v>131</v>
       </c>
       <c r="AM59" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN59" t="s" s="2">
-        <v>383</v>
+        <v>80</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
         <v>384</v>
       </c>
@@ -8498,7 +8597,7 @@
         <v>78</v>
       </c>
       <c r="G60" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H60" t="s" s="2">
         <v>80</v>
@@ -8510,7 +8609,7 @@
         <v>80</v>
       </c>
       <c r="K60" t="s" s="2">
-        <v>211</v>
+        <v>146</v>
       </c>
       <c r="L60" t="s" s="2">
         <v>385</v>
@@ -8518,12 +8617,8 @@
       <c r="M60" t="s" s="2">
         <v>386</v>
       </c>
-      <c r="N60" t="s" s="2">
-        <v>387</v>
-      </c>
-      <c r="O60" t="s" s="2">
-        <v>388</v>
-      </c>
+      <c r="N60" s="2"/>
+      <c r="O60" s="2"/>
       <c r="P60" t="s" s="2">
         <v>80</v>
       </c>
@@ -8547,13 +8642,13 @@
         <v>80</v>
       </c>
       <c r="X60" t="s" s="2">
-        <v>215</v>
+        <v>80</v>
       </c>
       <c r="Y60" t="s" s="2">
-        <v>389</v>
+        <v>80</v>
       </c>
       <c r="Z60" t="s" s="2">
-        <v>390</v>
+        <v>80</v>
       </c>
       <c r="AA60" t="s" s="2">
         <v>80</v>
@@ -8577,7 +8672,7 @@
         <v>78</v>
       </c>
       <c r="AH60" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI60" t="s" s="2">
         <v>80</v>
@@ -8589,21 +8684,21 @@
         <v>80</v>
       </c>
       <c r="AL60" t="s" s="2">
-        <v>391</v>
+        <v>150</v>
       </c>
       <c r="AM60" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN60" t="s" s="2">
-        <v>392</v>
+        <v>387</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="2">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -8614,10 +8709,10 @@
         <v>78</v>
       </c>
       <c r="G61" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H61" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I61" t="s" s="2">
         <v>80</v>
@@ -8626,13 +8721,13 @@
         <v>80</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>211</v>
+        <v>389</v>
       </c>
       <c r="L61" t="s" s="2">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="M61" t="s" s="2">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="N61" s="2"/>
       <c r="O61" s="2"/>
@@ -8659,13 +8754,13 @@
         <v>80</v>
       </c>
       <c r="X61" t="s" s="2">
-        <v>112</v>
+        <v>80</v>
       </c>
       <c r="Y61" t="s" s="2">
-        <v>396</v>
+        <v>80</v>
       </c>
       <c r="Z61" t="s" s="2">
-        <v>397</v>
+        <v>80</v>
       </c>
       <c r="AA61" t="s" s="2">
         <v>80</v>
@@ -8683,13 +8778,13 @@
         <v>80</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH61" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI61" t="s" s="2">
         <v>80</v>
@@ -8701,21 +8796,21 @@
         <v>80</v>
       </c>
       <c r="AL61" t="s" s="2">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="AM61" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN61" t="s" s="2">
-        <v>399</v>
+        <v>80</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>400</v>
+        <v>393</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>400</v>
+        <v>393</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -8726,7 +8821,7 @@
         <v>78</v>
       </c>
       <c r="G62" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H62" t="s" s="2">
         <v>80</v>
@@ -8741,10 +8836,10 @@
         <v>211</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>401</v>
+        <v>394</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>402</v>
+        <v>395</v>
       </c>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
@@ -8774,10 +8869,10 @@
         <v>112</v>
       </c>
       <c r="Y62" t="s" s="2">
-        <v>403</v>
+        <v>396</v>
       </c>
       <c r="Z62" t="s" s="2">
-        <v>404</v>
+        <v>397</v>
       </c>
       <c r="AA62" t="s" s="2">
         <v>80</v>
@@ -8795,13 +8890,13 @@
         <v>80</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>400</v>
+        <v>393</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH62" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI62" t="s" s="2">
         <v>80</v>
@@ -8813,21 +8908,21 @@
         <v>80</v>
       </c>
       <c r="AL62" t="s" s="2">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="AM62" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN62" t="s" s="2">
-        <v>406</v>
+        <v>399</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -8850,13 +8945,13 @@
         <v>80</v>
       </c>
       <c r="K63" t="s" s="2">
-        <v>367</v>
+        <v>211</v>
       </c>
       <c r="L63" t="s" s="2">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="M63" t="s" s="2">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="N63" s="2"/>
       <c r="O63" s="2"/>
@@ -8883,13 +8978,13 @@
         <v>80</v>
       </c>
       <c r="X63" t="s" s="2">
-        <v>80</v>
+        <v>215</v>
       </c>
       <c r="Y63" t="s" s="2">
-        <v>80</v>
+        <v>403</v>
       </c>
       <c r="Z63" t="s" s="2">
-        <v>80</v>
+        <v>404</v>
       </c>
       <c r="AA63" t="s" s="2">
         <v>80</v>
@@ -8907,7 +9002,7 @@
         <v>80</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>78</v>
@@ -8925,21 +9020,21 @@
         <v>80</v>
       </c>
       <c r="AL63" t="s" s="2">
-        <v>410</v>
+        <v>169</v>
       </c>
       <c r="AM63" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN63" t="s" s="2">
-        <v>411</v>
+        <v>405</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>412</v>
+        <v>406</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>412</v>
+        <v>406</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -8950,7 +9045,7 @@
         <v>78</v>
       </c>
       <c r="G64" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H64" t="s" s="2">
         <v>80</v>
@@ -8965,13 +9060,17 @@
         <v>211</v>
       </c>
       <c r="L64" t="s" s="2">
-        <v>413</v>
+        <v>407</v>
       </c>
       <c r="M64" t="s" s="2">
-        <v>414</v>
-      </c>
-      <c r="N64" s="2"/>
-      <c r="O64" s="2"/>
+        <v>408</v>
+      </c>
+      <c r="N64" t="s" s="2">
+        <v>409</v>
+      </c>
+      <c r="O64" t="s" s="2">
+        <v>410</v>
+      </c>
       <c r="P64" t="s" s="2">
         <v>80</v>
       </c>
@@ -8998,10 +9097,10 @@
         <v>215</v>
       </c>
       <c r="Y64" t="s" s="2">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="Z64" t="s" s="2">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="AA64" t="s" s="2">
         <v>80</v>
@@ -9019,13 +9118,13 @@
         <v>80</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>412</v>
+        <v>406</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH64" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI64" t="s" s="2">
         <v>80</v>
@@ -9037,21 +9136,21 @@
         <v>80</v>
       </c>
       <c r="AL64" t="s" s="2">
-        <v>417</v>
+        <v>413</v>
       </c>
       <c r="AM64" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN64" t="s" s="2">
-        <v>418</v>
+        <v>414</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -9074,17 +9173,15 @@
         <v>80</v>
       </c>
       <c r="K65" t="s" s="2">
-        <v>165</v>
+        <v>211</v>
       </c>
       <c r="L65" t="s" s="2">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="M65" t="s" s="2">
-        <v>421</v>
-      </c>
-      <c r="N65" t="s" s="2">
-        <v>422</v>
-      </c>
+        <v>417</v>
+      </c>
+      <c r="N65" s="2"/>
       <c r="O65" s="2"/>
       <c r="P65" t="s" s="2">
         <v>80</v>
@@ -9109,13 +9206,13 @@
         <v>80</v>
       </c>
       <c r="X65" t="s" s="2">
-        <v>80</v>
+        <v>112</v>
       </c>
       <c r="Y65" t="s" s="2">
-        <v>80</v>
+        <v>418</v>
       </c>
       <c r="Z65" t="s" s="2">
-        <v>80</v>
+        <v>419</v>
       </c>
       <c r="AA65" t="s" s="2">
         <v>80</v>
@@ -9133,7 +9230,7 @@
         <v>80</v>
       </c>
       <c r="AF65" t="s" s="2">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="AG65" t="s" s="2">
         <v>78</v>
@@ -9151,21 +9248,21 @@
         <v>80</v>
       </c>
       <c r="AL65" t="s" s="2">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="AM65" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN65" t="s" s="2">
-        <v>80</v>
+        <v>421</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -9176,7 +9273,7 @@
         <v>78</v>
       </c>
       <c r="G66" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H66" t="s" s="2">
         <v>80</v>
@@ -9188,13 +9285,13 @@
         <v>80</v>
       </c>
       <c r="K66" t="s" s="2">
-        <v>171</v>
+        <v>211</v>
       </c>
       <c r="L66" t="s" s="2">
-        <v>172</v>
+        <v>423</v>
       </c>
       <c r="M66" t="s" s="2">
-        <v>173</v>
+        <v>424</v>
       </c>
       <c r="N66" s="2"/>
       <c r="O66" s="2"/>
@@ -9221,13 +9318,13 @@
         <v>80</v>
       </c>
       <c r="X66" t="s" s="2">
-        <v>80</v>
+        <v>112</v>
       </c>
       <c r="Y66" t="s" s="2">
-        <v>80</v>
+        <v>425</v>
       </c>
       <c r="Z66" t="s" s="2">
-        <v>80</v>
+        <v>426</v>
       </c>
       <c r="AA66" t="s" s="2">
         <v>80</v>
@@ -9245,50 +9342,50 @@
         <v>80</v>
       </c>
       <c r="AF66" t="s" s="2">
-        <v>174</v>
+        <v>422</v>
       </c>
       <c r="AG66" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH66" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI66" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ66" t="s" s="2">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="AK66" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL66" t="s" s="2">
-        <v>169</v>
+        <v>427</v>
       </c>
       <c r="AM66" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN66" t="s" s="2">
-        <v>80</v>
+        <v>428</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" hidden="true">
       <c r="A67" t="s" s="2">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
-        <v>133</v>
+        <v>80</v>
       </c>
       <c r="E67" s="2"/>
       <c r="F67" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G67" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H67" t="s" s="2">
         <v>80</v>
@@ -9300,17 +9397,15 @@
         <v>80</v>
       </c>
       <c r="K67" t="s" s="2">
-        <v>134</v>
+        <v>430</v>
       </c>
       <c r="L67" t="s" s="2">
-        <v>135</v>
+        <v>431</v>
       </c>
       <c r="M67" t="s" s="2">
-        <v>176</v>
-      </c>
-      <c r="N67" t="s" s="2">
-        <v>137</v>
-      </c>
+        <v>432</v>
+      </c>
+      <c r="N67" s="2"/>
       <c r="O67" s="2"/>
       <c r="P67" t="s" s="2">
         <v>80</v>
@@ -9359,75 +9454,71 @@
         <v>80</v>
       </c>
       <c r="AF67" t="s" s="2">
-        <v>177</v>
+        <v>429</v>
       </c>
       <c r="AG67" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH67" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI67" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ67" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK67" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL67" t="s" s="2">
-        <v>169</v>
+        <v>433</v>
       </c>
       <c r="AM67" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN67" t="s" s="2">
-        <v>80</v>
+        <v>434</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s" s="2">
-        <v>426</v>
+        <v>435</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>426</v>
+        <v>435</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
-        <v>179</v>
+        <v>80</v>
       </c>
       <c r="E68" s="2"/>
       <c r="F68" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G68" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H68" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I68" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="J68" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K68" t="s" s="2">
-        <v>134</v>
+        <v>211</v>
       </c>
       <c r="L68" t="s" s="2">
-        <v>180</v>
+        <v>436</v>
       </c>
       <c r="M68" t="s" s="2">
-        <v>181</v>
-      </c>
-      <c r="N68" t="s" s="2">
-        <v>137</v>
-      </c>
-      <c r="O68" t="s" s="2">
-        <v>143</v>
-      </c>
+        <v>437</v>
+      </c>
+      <c r="N68" s="2"/>
+      <c r="O68" s="2"/>
       <c r="P68" t="s" s="2">
         <v>80</v>
       </c>
@@ -9451,13 +9542,13 @@
         <v>80</v>
       </c>
       <c r="X68" t="s" s="2">
-        <v>80</v>
+        <v>215</v>
       </c>
       <c r="Y68" t="s" s="2">
-        <v>80</v>
+        <v>438</v>
       </c>
       <c r="Z68" t="s" s="2">
-        <v>80</v>
+        <v>439</v>
       </c>
       <c r="AA68" t="s" s="2">
         <v>80</v>
@@ -9475,39 +9566,39 @@
         <v>80</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>182</v>
+        <v>435</v>
       </c>
       <c r="AG68" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH68" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI68" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ68" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK68" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL68" t="s" s="2">
-        <v>131</v>
+        <v>440</v>
       </c>
       <c r="AM68" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN68" t="s" s="2">
-        <v>80</v>
+        <v>441</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
-        <v>427</v>
+        <v>442</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>427</v>
+        <v>442</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -9515,13 +9606,13 @@
       </c>
       <c r="E69" s="2"/>
       <c r="F69" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G69" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H69" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I69" t="s" s="2">
         <v>80</v>
@@ -9530,15 +9621,17 @@
         <v>80</v>
       </c>
       <c r="K69" t="s" s="2">
-        <v>428</v>
+        <v>165</v>
       </c>
       <c r="L69" t="s" s="2">
-        <v>429</v>
+        <v>443</v>
       </c>
       <c r="M69" t="s" s="2">
-        <v>430</v>
-      </c>
-      <c r="N69" s="2"/>
+        <v>444</v>
+      </c>
+      <c r="N69" t="s" s="2">
+        <v>445</v>
+      </c>
       <c r="O69" s="2"/>
       <c r="P69" t="s" s="2">
         <v>80</v>
@@ -9587,13 +9680,13 @@
         <v>80</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>427</v>
+        <v>442</v>
       </c>
       <c r="AG69" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="AH69" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI69" t="s" s="2">
         <v>80</v>
@@ -9602,24 +9695,24 @@
         <v>100</v>
       </c>
       <c r="AK69" t="s" s="2">
-        <v>431</v>
+        <v>80</v>
       </c>
       <c r="AL69" t="s" s="2">
-        <v>285</v>
+        <v>446</v>
       </c>
       <c r="AM69" t="s" s="2">
-        <v>432</v>
+        <v>80</v>
       </c>
       <c r="AN69" t="s" s="2">
-        <v>433</v>
+        <v>80</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" hidden="true">
       <c r="A70" t="s" s="2">
-        <v>434</v>
+        <v>447</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>434</v>
+        <v>447</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -9642,17 +9735,15 @@
         <v>80</v>
       </c>
       <c r="K70" t="s" s="2">
-        <v>108</v>
+        <v>171</v>
       </c>
       <c r="L70" t="s" s="2">
-        <v>435</v>
+        <v>172</v>
       </c>
       <c r="M70" t="s" s="2">
-        <v>436</v>
-      </c>
-      <c r="N70" t="s" s="2">
-        <v>437</v>
-      </c>
+        <v>173</v>
+      </c>
+      <c r="N70" s="2"/>
       <c r="O70" s="2"/>
       <c r="P70" t="s" s="2">
         <v>80</v>
@@ -9677,13 +9768,13 @@
         <v>80</v>
       </c>
       <c r="X70" t="s" s="2">
-        <v>157</v>
+        <v>80</v>
       </c>
       <c r="Y70" t="s" s="2">
-        <v>438</v>
+        <v>80</v>
       </c>
       <c r="Z70" t="s" s="2">
-        <v>439</v>
+        <v>80</v>
       </c>
       <c r="AA70" t="s" s="2">
         <v>80</v>
@@ -9701,7 +9792,7 @@
         <v>80</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>434</v>
+        <v>174</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>78</v>
@@ -9713,13 +9804,13 @@
         <v>80</v>
       </c>
       <c r="AJ70" t="s" s="2">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AK70" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL70" t="s" s="2">
-        <v>440</v>
+        <v>169</v>
       </c>
       <c r="AM70" t="s" s="2">
         <v>80</v>
@@ -9728,23 +9819,23 @@
         <v>80</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" hidden="true">
       <c r="A71" t="s" s="2">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
-        <v>80</v>
+        <v>133</v>
       </c>
       <c r="E71" s="2"/>
       <c r="F71" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G71" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H71" t="s" s="2">
         <v>80</v>
@@ -9756,16 +9847,16 @@
         <v>80</v>
       </c>
       <c r="K71" t="s" s="2">
-        <v>211</v>
+        <v>134</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>442</v>
+        <v>135</v>
       </c>
       <c r="M71" t="s" s="2">
-        <v>443</v>
+        <v>176</v>
       </c>
       <c r="N71" t="s" s="2">
-        <v>444</v>
+        <v>137</v>
       </c>
       <c r="O71" s="2"/>
       <c r="P71" t="s" s="2">
@@ -9791,13 +9882,13 @@
         <v>80</v>
       </c>
       <c r="X71" t="s" s="2">
-        <v>215</v>
+        <v>80</v>
       </c>
       <c r="Y71" t="s" s="2">
-        <v>445</v>
+        <v>80</v>
       </c>
       <c r="Z71" t="s" s="2">
-        <v>446</v>
+        <v>80</v>
       </c>
       <c r="AA71" t="s" s="2">
         <v>80</v>
@@ -9815,25 +9906,25 @@
         <v>80</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>441</v>
+        <v>177</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH71" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI71" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ71" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK71" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL71" t="s" s="2">
-        <v>80</v>
+        <v>169</v>
       </c>
       <c r="AM71" t="s" s="2">
         <v>80</v>
@@ -9842,44 +9933,48 @@
         <v>80</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" hidden="true">
       <c r="A72" t="s" s="2">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
-        <v>80</v>
+        <v>179</v>
       </c>
       <c r="E72" s="2"/>
       <c r="F72" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G72" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H72" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I72" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="J72" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K72" t="s" s="2">
-        <v>185</v>
+        <v>134</v>
       </c>
       <c r="L72" t="s" s="2">
-        <v>448</v>
+        <v>180</v>
       </c>
       <c r="M72" t="s" s="2">
-        <v>449</v>
-      </c>
-      <c r="N72" s="2"/>
-      <c r="O72" s="2"/>
+        <v>181</v>
+      </c>
+      <c r="N72" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="O72" t="s" s="2">
+        <v>143</v>
+      </c>
       <c r="P72" t="s" s="2">
         <v>80</v>
       </c>
@@ -9927,25 +10022,25 @@
         <v>80</v>
       </c>
       <c r="AF72" t="s" s="2">
-        <v>447</v>
+        <v>182</v>
       </c>
       <c r="AG72" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH72" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI72" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ72" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK72" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL72" t="s" s="2">
-        <v>278</v>
+        <v>131</v>
       </c>
       <c r="AM72" t="s" s="2">
         <v>80</v>
@@ -9967,13 +10062,13 @@
       </c>
       <c r="E73" s="2"/>
       <c r="F73" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G73" t="s" s="2">
         <v>88</v>
       </c>
       <c r="H73" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I73" t="s" s="2">
         <v>80</v>
@@ -10042,7 +10137,7 @@
         <v>450</v>
       </c>
       <c r="AG73" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="AH73" t="s" s="2">
         <v>88</v>
@@ -10054,24 +10149,24 @@
         <v>100</v>
       </c>
       <c r="AK73" t="s" s="2">
-        <v>284</v>
+        <v>454</v>
       </c>
       <c r="AL73" t="s" s="2">
-        <v>454</v>
+        <v>285</v>
       </c>
       <c r="AM73" t="s" s="2">
-        <v>80</v>
+        <v>455</v>
       </c>
       <c r="AN73" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" hidden="true">
       <c r="A74" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -10094,7 +10189,7 @@
         <v>80</v>
       </c>
       <c r="K74" t="s" s="2">
-        <v>457</v>
+        <v>108</v>
       </c>
       <c r="L74" t="s" s="2">
         <v>458</v>
@@ -10129,13 +10224,13 @@
         <v>80</v>
       </c>
       <c r="X74" t="s" s="2">
-        <v>80</v>
+        <v>157</v>
       </c>
       <c r="Y74" t="s" s="2">
-        <v>80</v>
+        <v>461</v>
       </c>
       <c r="Z74" t="s" s="2">
-        <v>80</v>
+        <v>462</v>
       </c>
       <c r="AA74" t="s" s="2">
         <v>80</v>
@@ -10153,7 +10248,7 @@
         <v>80</v>
       </c>
       <c r="AF74" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="AG74" t="s" s="2">
         <v>78</v>
@@ -10168,19 +10263,489 @@
         <v>100</v>
       </c>
       <c r="AK74" t="s" s="2">
-        <v>461</v>
+        <v>80</v>
       </c>
       <c r="AL74" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="AM74" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN74" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="75" hidden="true">
+      <c r="A75" t="s" s="2">
+        <v>464</v>
+      </c>
+      <c r="B75" t="s" s="2">
+        <v>464</v>
+      </c>
+      <c r="C75" s="2"/>
+      <c r="D75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E75" s="2"/>
+      <c r="F75" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G75" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="H75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K75" t="s" s="2">
+        <v>211</v>
+      </c>
+      <c r="L75" t="s" s="2">
+        <v>465</v>
+      </c>
+      <c r="M75" t="s" s="2">
+        <v>466</v>
+      </c>
+      <c r="N75" t="s" s="2">
+        <v>467</v>
+      </c>
+      <c r="O75" s="2"/>
+      <c r="P75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q75" s="2"/>
+      <c r="R75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X75" t="s" s="2">
+        <v>215</v>
+      </c>
+      <c r="Y75" t="s" s="2">
+        <v>468</v>
+      </c>
+      <c r="Z75" t="s" s="2">
+        <v>469</v>
+      </c>
+      <c r="AA75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF75" t="s" s="2">
+        <v>464</v>
+      </c>
+      <c r="AG75" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH75" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ75" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM75" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN75" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="76" hidden="true">
+      <c r="A76" t="s" s="2">
+        <v>470</v>
+      </c>
+      <c r="B76" t="s" s="2">
+        <v>470</v>
+      </c>
+      <c r="C76" s="2"/>
+      <c r="D76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E76" s="2"/>
+      <c r="F76" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G76" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="H76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K76" t="s" s="2">
+        <v>185</v>
+      </c>
+      <c r="L76" t="s" s="2">
+        <v>471</v>
+      </c>
+      <c r="M76" t="s" s="2">
+        <v>472</v>
+      </c>
+      <c r="N76" s="2"/>
+      <c r="O76" s="2"/>
+      <c r="P76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q76" s="2"/>
+      <c r="R76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF76" t="s" s="2">
+        <v>470</v>
+      </c>
+      <c r="AG76" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH76" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ76" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL76" t="s" s="2">
+        <v>278</v>
+      </c>
+      <c r="AM76" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN76" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="s" s="2">
+        <v>473</v>
+      </c>
+      <c r="B77" t="s" s="2">
+        <v>473</v>
+      </c>
+      <c r="C77" s="2"/>
+      <c r="D77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E77" s="2"/>
+      <c r="F77" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G77" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="H77" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="I77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K77" t="s" s="2">
+        <v>474</v>
+      </c>
+      <c r="L77" t="s" s="2">
+        <v>475</v>
+      </c>
+      <c r="M77" t="s" s="2">
+        <v>476</v>
+      </c>
+      <c r="N77" s="2"/>
+      <c r="O77" s="2"/>
+      <c r="P77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q77" s="2"/>
+      <c r="R77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF77" t="s" s="2">
+        <v>473</v>
+      </c>
+      <c r="AG77" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH77" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ77" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK77" t="s" s="2">
+        <v>284</v>
+      </c>
+      <c r="AL77" t="s" s="2">
+        <v>477</v>
+      </c>
+      <c r="AM77" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN77" t="s" s="2">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="78" hidden="true">
+      <c r="A78" t="s" s="2">
+        <v>479</v>
+      </c>
+      <c r="B78" t="s" s="2">
+        <v>479</v>
+      </c>
+      <c r="C78" s="2"/>
+      <c r="D78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E78" s="2"/>
+      <c r="F78" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G78" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="H78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K78" t="s" s="2">
+        <v>480</v>
+      </c>
+      <c r="L78" t="s" s="2">
+        <v>481</v>
+      </c>
+      <c r="M78" t="s" s="2">
+        <v>482</v>
+      </c>
+      <c r="N78" t="s" s="2">
+        <v>483</v>
+      </c>
+      <c r="O78" s="2"/>
+      <c r="P78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q78" s="2"/>
+      <c r="R78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF78" t="s" s="2">
+        <v>479</v>
+      </c>
+      <c r="AG78" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH78" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ78" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK78" t="s" s="2">
+        <v>484</v>
+      </c>
+      <c r="AL78" t="s" s="2">
+        <v>485</v>
+      </c>
+      <c r="AM78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN78" t="s" s="2">
         <v>80</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AN78">
+    <filterColumn colId="7">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+    <filterColumn colId="27">
+      <filters blank="true"/>
+    </filterColumn>
+  </autoFilter>
+  <conditionalFormatting sqref="A2:AI77">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>$G2&lt;&gt;"Y"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>$Q2&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>